<commit_message>
Added new 2022 metadata to all porewater file
</commit_message>
<xml_diff>
--- a/processing_scripts/Inventory_Processing/2022 Metadata Creation/Source_Water_Metadata_Jun2022_Event.xlsx
+++ b/processing_scripts/Inventory_Processing/2022 Metadata Creation/Source_Water_Metadata_Jun2022_Event.xlsx
@@ -13,10 +13,10 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author>tc={29d6b5ec-fca1-468f-97bf-0c5a0eb2c86d}</author>
+    <author>tc={15fd8c64-760b-4609-a465-bc539c666136}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{29d6b5ec-fca1-468f-97bf-0c5a0eb2c86d}" ref="D14">
+    <comment authorId="0" xr:uid="{15fd8c64-760b-4609-a465-bc539c666136}" ref="D14">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -260,9 +260,9 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <x18tc:person displayName="opal.otenburg@gmail.com" id="{94bfc595-5d66-40e0-9d06-18f453d17c60}" userId="opal.otenburg@gmail.com" providerId="google-sheets"/>
-  <x18tc:person displayName="opal.otenburg@pnnl.gov" id="{b64bcd72-58a9-4e86-85bb-b7572a145765}" userId="opal.otenburg@pnnl.gov" providerId="google-sheets"/>
-  <x18tc:person displayName="Allison Myers-Pigg" id="{ea4c3fc4-3a7f-4232-a0a5-3e9509bf8699}" providerId="google-sheets"/>
+  <x18tc:person displayName="opal.otenburg@gmail.com" id="{f341c72f-06c0-4319-aa21-88a8230b84ae}" userId="opal.otenburg@gmail.com" providerId="google-sheets"/>
+  <x18tc:person displayName="opal.otenburg@pnnl.gov" id="{6e2c629d-8904-4e8f-b364-348e79d803c9}" userId="opal.otenburg@pnnl.gov" providerId="google-sheets"/>
+  <x18tc:person displayName="Allison Myers-Pigg" id="{9357c7c9-9eaa-4b95-a81b-bc8ac4130609}" providerId="google-sheets"/>
 </x18tc:personList>
 </file>
 
@@ -462,14 +462,14 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="D14" dT="2022-06-25T11:02:04.00" personId="{ea4c3fc4-3a7f-4232-a0a5-3e9509bf8699}" id="{29d6b5ec-fca1-468f-97bf-0c5a0eb2c86d}" done="0">
+  <x18tc:threadedComment ref="D14" dT="2022-06-25T11:02:04.00" personId="{9357c7c9-9eaa-4b95-a81b-bc8ac4130609}" id="{15fd8c64-760b-4609-a465-bc539c666136}" done="0">
     <x18tc:text xml:space="preserve">@opal.otenburg@gmail.com @opal.otenburg@pnnl.gov  Were these vials corrected? If so, please also correct this column. thanks!</x18tc:text>
     <x18tc:mentions>
-      <x18tc:mention mentionpersonId="{94bfc595-5d66-40e0-9d06-18f453d17c60}" mentionId="{1be4509c-cd85-499c-bd8c-cff07d1b3a1b}" startIndex="0" length="24"/>
-      <x18tc:mention mentionpersonId="{b64bcd72-58a9-4e86-85bb-b7572a145765}" mentionId="{f9dfce5d-45b6-4909-a971-eaaa9ec197f4}" startIndex="25" length="23"/>
+      <x18tc:mention mentionpersonId="{f341c72f-06c0-4319-aa21-88a8230b84ae}" mentionId="{4708a1d8-fe3c-4c8d-9ee2-8a6240f28c94}" startIndex="0" length="24"/>
+      <x18tc:mention mentionpersonId="{6e2c629d-8904-4e8f-b364-348e79d803c9}" mentionId="{486387ee-c2b4-401b-a7cd-c99b342412ec}" startIndex="25" length="23"/>
     </x18tc:mentions>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="D14" dT="2022-07-08T16:08:56.00" personId="{ea4c3fc4-3a7f-4232-a0a5-3e9509bf8699}" id="{85850a1e-8297-4ebe-925e-19c6aef1dc6a}" parentId="{29d6b5ec-fca1-468f-97bf-0c5a0eb2c86d}">
+  <x18tc:threadedComment ref="D14" dT="2022-07-08T16:08:56.00" personId="{9357c7c9-9eaa-4b95-a81b-bc8ac4130609}" id="{101229df-feb2-405b-94f2-8683a86f4d0f}" parentId="{15fd8c64-760b-4609-a465-bc539c666136}">
     <x18tc:text xml:space="preserve">Change from Hr 6 to Hr 7</x18tc:text>
   </x18tc:threadedComment>
 </x18tc:ThreadedComments>

</xml_diff>

<commit_message>
Fixed times for porewater data
</commit_message>
<xml_diff>
--- a/processing_scripts/Inventory_Processing/2022 Metadata Creation/Source_Water_Metadata_Jun2022_Event.xlsx
+++ b/processing_scripts/Inventory_Processing/2022 Metadata Creation/Source_Water_Metadata_Jun2022_Event.xlsx
@@ -13,10 +13,10 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author>tc={15fd8c64-760b-4609-a465-bc539c666136}</author>
+    <author>tc={65deb527-f365-4bb3-89b0-40f0d7ffd40f}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{15fd8c64-760b-4609-a465-bc539c666136}" ref="D14">
+    <comment authorId="0" xr:uid="{65deb527-f365-4bb3-89b0-40f0d7ffd40f}" ref="D14">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -260,9 +260,9 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <x18tc:person displayName="opal.otenburg@gmail.com" id="{f341c72f-06c0-4319-aa21-88a8230b84ae}" userId="opal.otenburg@gmail.com" providerId="google-sheets"/>
-  <x18tc:person displayName="opal.otenburg@pnnl.gov" id="{6e2c629d-8904-4e8f-b364-348e79d803c9}" userId="opal.otenburg@pnnl.gov" providerId="google-sheets"/>
-  <x18tc:person displayName="Allison Myers-Pigg" id="{9357c7c9-9eaa-4b95-a81b-bc8ac4130609}" providerId="google-sheets"/>
+  <x18tc:person displayName="opal.otenburg@gmail.com" id="{8b086c0f-aa38-4d93-af6b-fc644314277a}" userId="opal.otenburg@gmail.com" providerId="google-sheets"/>
+  <x18tc:person displayName="opal.otenburg@pnnl.gov" id="{ca70ef68-a66b-447c-a79a-33eefce2e60f}" userId="opal.otenburg@pnnl.gov" providerId="google-sheets"/>
+  <x18tc:person displayName="Allison Myers-Pigg" id="{884b0f02-3bf0-41be-b150-5560e8dd3975}" providerId="google-sheets"/>
 </x18tc:personList>
 </file>
 
@@ -462,14 +462,14 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="D14" dT="2022-06-25T11:02:04.00" personId="{9357c7c9-9eaa-4b95-a81b-bc8ac4130609}" id="{15fd8c64-760b-4609-a465-bc539c666136}" done="0">
+  <x18tc:threadedComment ref="D14" dT="2022-06-25T11:02:04.00" personId="{884b0f02-3bf0-41be-b150-5560e8dd3975}" id="{65deb527-f365-4bb3-89b0-40f0d7ffd40f}" done="0">
     <x18tc:text xml:space="preserve">@opal.otenburg@gmail.com @opal.otenburg@pnnl.gov  Were these vials corrected? If so, please also correct this column. thanks!</x18tc:text>
     <x18tc:mentions>
-      <x18tc:mention mentionpersonId="{f341c72f-06c0-4319-aa21-88a8230b84ae}" mentionId="{4708a1d8-fe3c-4c8d-9ee2-8a6240f28c94}" startIndex="0" length="24"/>
-      <x18tc:mention mentionpersonId="{6e2c629d-8904-4e8f-b364-348e79d803c9}" mentionId="{486387ee-c2b4-401b-a7cd-c99b342412ec}" startIndex="25" length="23"/>
+      <x18tc:mention mentionpersonId="{8b086c0f-aa38-4d93-af6b-fc644314277a}" mentionId="{9e858b59-ac10-4fc1-afde-9d407784c5ec}" startIndex="0" length="24"/>
+      <x18tc:mention mentionpersonId="{ca70ef68-a66b-447c-a79a-33eefce2e60f}" mentionId="{35fac549-bd99-4abc-b944-f4f336f07468}" startIndex="25" length="23"/>
     </x18tc:mentions>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="D14" dT="2022-07-08T16:08:56.00" personId="{9357c7c9-9eaa-4b95-a81b-bc8ac4130609}" id="{101229df-feb2-405b-94f2-8683a86f4d0f}" parentId="{15fd8c64-760b-4609-a465-bc539c666136}">
+  <x18tc:threadedComment ref="D14" dT="2022-07-08T16:08:56.00" personId="{884b0f02-3bf0-41be-b150-5560e8dd3975}" id="{ececfb02-95a0-48a7-8360-951fcbf8d013}" parentId="{65deb527-f365-4bb3-89b0-40f0d7ffd40f}">
     <x18tc:text xml:space="preserve">Change from Hr 6 to Hr 7</x18tc:text>
   </x18tc:threadedComment>
 </x18tc:ThreadedComments>

</xml_diff>